<commit_message>
Update Egen_analys.xlsx for internal analysis
- Updated the existing Egen_analys.xlsx file to reflect recent changes and improvements in internal analysis processes for Kalmar Nation.
- This update aims to enhance data accuracy and support more effective decision-making within the organization.
</commit_message>
<xml_diff>
--- a/KalmarNation/revision/_egen_analys/Egen_analys.xlsx
+++ b/KalmarNation/revision/_egen_analys/Egen_analys.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/ClaudeCowork/KalmarNation/revision/_egen_analys/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{CFF8497D-5AC5-4F53-BB79-950D853A1C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AD9A71D-6F8F-4F48-A60D-7A52B8BBFD63}"/>
+  <xr:revisionPtr revIDLastSave="238" documentId="8_{CFF8497D-5AC5-4F53-BB79-950D853A1C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80CAC469-ADE8-49DF-9C28-AF10224B0F30}"/>
   <bookViews>
-    <workbookView xWindow="-21450" yWindow="2190" windowWidth="21600" windowHeight="11295" xr2:uid="{3C2F71A7-BF18-485F-8BF5-EA2F93EB7B3B}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3C2F71A7-BF18-485F-8BF5-EA2F93EB7B3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="39">
   <si>
     <t>Resultat efter finansiella poster:</t>
   </si>
@@ -55,13 +55,109 @@
   </si>
   <si>
     <t>kr</t>
+  </si>
+  <si>
+    <t>IB</t>
+  </si>
+  <si>
+    <t>förändring</t>
+  </si>
+  <si>
+    <t>UB</t>
+  </si>
+  <si>
+    <t>Summa eget kapital:</t>
+  </si>
+  <si>
+    <t>Beräknat resultat:</t>
+  </si>
+  <si>
+    <t>Jag vill att det egna kapitalet ska öka med resultatet</t>
+  </si>
+  <si>
+    <t>Summa eget kapital och skulder:</t>
+  </si>
+  <si>
+    <t>Övriga skulder:</t>
+  </si>
+  <si>
+    <t>Differnas mot Summa tillgångar (10 055 854 kr):</t>
+  </si>
+  <si>
+    <t>Nu ser skulderna ut så här</t>
+  </si>
+  <si>
+    <t>Kommentar</t>
+  </si>
+  <si>
+    <t>Summa eget kapital, kto 2010:</t>
+  </si>
+  <si>
+    <t>Summa eget kapital (kto 2010 och 2099):</t>
+  </si>
+  <si>
+    <t>Förslag på förändring av eget kapital</t>
+  </si>
+  <si>
+    <t>IB 2025</t>
+  </si>
+  <si>
+    <t>UB 2025</t>
+  </si>
+  <si>
+    <t>Beskrivning</t>
+  </si>
+  <si>
+    <t>Årets överskott</t>
+  </si>
+  <si>
+    <t>Summa disponibelt</t>
+  </si>
+  <si>
+    <t>Belopp (kr)</t>
+  </si>
+  <si>
+    <t>Till förfogande står följande medel:</t>
+  </si>
+  <si>
+    <t>Balanserat överskott (ingående)</t>
+  </si>
+  <si>
+    <t>som är lagerförändringar 2025</t>
+  </si>
+  <si>
+    <t>Rätt resultat 2025 enligt Kent</t>
+  </si>
+  <si>
+    <t>Lagerförändringar:</t>
+  </si>
+  <si>
+    <t>Men resultat är ju 434 975 kr</t>
+  </si>
+  <si>
+    <t>inklusive lagerförändringa om 15 929 kr</t>
+  </si>
+  <si>
+    <t>Årets (2025) resultat, kto 2099:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Styrelsen föreslår följande disposition: </t>
+  </si>
+  <si>
+    <t>Årets överskott om 434 975 kr överförs i sin helhet till balanserat överskott.</t>
+  </si>
+  <si>
+    <t>FÖRSLAG TILL VINSTDISPOSITION</t>
+  </si>
+  <si>
+    <t>När årsmötet har godkänt dispositionen så bokförs debet konto 2099 Åres resultat 434 975 kr, och kredit konto 2010 summa eget kapital.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -77,13 +173,34 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -98,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -113,6 +230,57 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -427,43 +595,67 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F70D926-ACEA-4DAF-A8D9-1FE06F404D0C}">
-  <dimension ref="J3:N27"/>
+  <dimension ref="B3:N45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="42.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="43.42578125" customWidth="1"/>
     <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="L4" s="2"/>
       <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="L5" s="2"/>
       <c r="M5" s="1">
         <v>1316632</v>
       </c>
     </row>
-    <row r="6" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="L6" s="2"/>
       <c r="M6" s="1">
         <v>881657</v>
       </c>
     </row>
-    <row r="7" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="L7" s="2"/>
       <c r="M7" s="1">
         <f>M5-M6</f>
         <v>434975</v>
       </c>
     </row>
-    <row r="8" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="E8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="1"/>
     </row>
-    <row r="9" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="L9" s="2" t="s">
         <v>5</v>
       </c>
@@ -471,7 +663,24 @@
         <v>1300704</v>
       </c>
     </row>
-    <row r="10" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B10" s="11"/>
+      <c r="C10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="E10" s="19">
+        <v>881657</v>
+      </c>
+      <c r="F10" s="12">
+        <f>D10+E10</f>
+        <v>-8626036</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>6</v>
+      </c>
       <c r="L10" s="2" t="s">
         <v>1</v>
       </c>
@@ -479,7 +688,13 @@
         <v>-881657</v>
       </c>
     </row>
-    <row r="11" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B11" s="11"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
       <c r="L11" s="2" t="s">
         <v>0</v>
       </c>
@@ -488,37 +703,95 @@
         <v>419047</v>
       </c>
     </row>
-    <row r="12" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B12" s="11"/>
+      <c r="C12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="12"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="12">
+        <f>1316633</f>
+        <v>1316633</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
       <c r="L12" s="2"/>
       <c r="M12" s="1"/>
     </row>
-    <row r="13" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C13" s="2"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
       <c r="L13" s="2"/>
       <c r="M13" s="4"/>
     </row>
-    <row r="14" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C14" s="2"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
       <c r="L14" s="3" t="s">
         <v>2</v>
       </c>
       <c r="M14" s="4">
-        <v>35303</v>
+        <v>35303.4</v>
       </c>
       <c r="N14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" s="12"/>
       <c r="L15" s="2" t="s">
         <v>3</v>
       </c>
       <c r="M15" s="4">
-        <v>578936</v>
+        <v>578936.24</v>
       </c>
       <c r="N15" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="12:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B16" s="11"/>
+      <c r="C16" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="E16" s="19">
+        <f>-F18</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="F16" s="12">
+        <f>D16+E16</f>
+        <v>-9942668.3699999992</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>6</v>
+      </c>
       <c r="L16" s="2" t="s">
         <v>4</v>
       </c>
@@ -529,70 +802,385 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="6" t="s">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B17" s="11"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="L17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M17" s="4">
+        <v>15928.73</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B18" s="11"/>
+      <c r="C18" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="12"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="12">
+        <f>M18</f>
+        <v>434975.37</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" t="s">
+        <v>30</v>
+      </c>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="M17" s="7">
-        <f>SUM(M14:M16)</f>
-        <v>419046</v>
-      </c>
-      <c r="N17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="L19" s="2" t="s">
+      <c r="M18" s="7">
+        <f>SUM(M14:M17)</f>
+        <v>434975.37</v>
+      </c>
+      <c r="N18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C19" s="2"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="25"/>
+      <c r="D20" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E20" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="12"/>
+      <c r="H20" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B21" s="8"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="12"/>
+      <c r="L21" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="M19" s="4">
+      <c r="M21" s="4">
         <v>881657</v>
       </c>
-      <c r="N19" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="L20" s="2" t="s">
+      <c r="N21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B22" s="11"/>
+      <c r="C22" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="E22" s="19">
+        <v>0</v>
+      </c>
+      <c r="F22" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L22" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="M20" s="4">
-        <f>SUM(M17:M19)</f>
-        <v>1300703</v>
-      </c>
-      <c r="N20" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="L21" s="2"/>
-      <c r="M21" s="4"/>
-    </row>
-    <row r="22" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="L22" s="2"/>
-      <c r="M22" s="4"/>
-    </row>
-    <row r="23" spans="10:14" x14ac:dyDescent="0.25">
+      <c r="M22" s="4">
+        <f>SUM(M18:M21)</f>
+        <v>1316632.3700000001</v>
+      </c>
+      <c r="N22" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B23" s="11"/>
+      <c r="C23" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="12">
+        <v>0</v>
+      </c>
+      <c r="E23" s="21">
+        <f>-F18</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="F23" s="12">
+        <f>D23+E23</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H23" t="s">
+        <v>33</v>
+      </c>
       <c r="L23" s="2"/>
       <c r="M23" s="4"/>
     </row>
-    <row r="24" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B24" s="11"/>
+      <c r="C24" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="14">
+        <f>SUM(D22:D23)</f>
+        <v>-9507693</v>
+      </c>
+      <c r="E24" s="14">
+        <f>SUM(E22:E23)</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="F24" s="14">
+        <f>SUM(F22:F23)</f>
+        <v>-9942668.3699999992</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>6</v>
+      </c>
       <c r="L24" s="2"/>
       <c r="M24" s="4"/>
     </row>
-    <row r="25" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B25" s="11"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="12"/>
       <c r="L25" s="2"/>
       <c r="M25" s="4"/>
     </row>
-    <row r="26" spans="10:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B26" s="11"/>
+      <c r="C26" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="12"/>
       <c r="L26" s="2"/>
-    </row>
-    <row r="27" spans="10:14" x14ac:dyDescent="0.25">
+      <c r="M26" s="4"/>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B27" s="11"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="12"/>
       <c r="L27" s="2"/>
+      <c r="M27" s="4"/>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B28" s="11"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="12"/>
+      <c r="L28" s="2"/>
+      <c r="M28" s="4"/>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B29" s="11"/>
+      <c r="C29" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="12"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="12">
+        <f>-113186</f>
+        <v>-113186</v>
+      </c>
+      <c r="G29" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L29" s="2"/>
+      <c r="M29" s="4"/>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B30" s="11"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="L30" s="2"/>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B31" s="11"/>
+      <c r="C31" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="14">
+        <f>SUM(F24:F30)</f>
+        <v>-10055854.369999999</v>
+      </c>
+      <c r="G31" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L31" s="2"/>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B32" s="16"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="16"/>
+    </row>
+    <row r="33" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="11"/>
+      <c r="C33" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="12">
+        <f>10055854+F31</f>
+        <v>-0.36999999918043613</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H33" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B35" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
+    </row>
+    <row r="36" spans="2:8" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="15"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+    </row>
+    <row r="37" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B37" s="11"/>
+      <c r="C37" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+    </row>
+    <row r="38" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="11"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="11"/>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B39" s="11"/>
+      <c r="C39" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D39" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="E39" s="11"/>
+      <c r="F39" s="11"/>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B40" s="11"/>
+      <c r="C40" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40" s="12">
+        <v>9507693</v>
+      </c>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B41" s="11"/>
+      <c r="C41" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" s="12">
+        <f>F18</f>
+        <v>434975.37</v>
+      </c>
+      <c r="E41" s="11"/>
+      <c r="F41" s="11"/>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B42" s="11"/>
+      <c r="C42" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D42" s="14">
+        <f>SUM(D40:D41)</f>
+        <v>9942668.3699999992</v>
+      </c>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B43" s="11"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="11"/>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B44" s="11"/>
+      <c r="C44" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="11"/>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B45" s="11"/>
+      <c r="C45" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="11"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C26:F27"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add financial reports for 2025 and 2026, including Balansrapport and Resultatrapport. Updated document versions to reflect the latest financial data as of 2026-04-27. Ensured consistency across all reports for accurate financial tracking and compliance.
</commit_message>
<xml_diff>
--- a/KalmarNation/revision/_egen_analys/Egen_analys.xlsx
+++ b/KalmarNation/revision/_egen_analys/Egen_analys.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/ClaudeCowork/KalmarNation/revision/_egen_analys/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="238" documentId="8_{CFF8497D-5AC5-4F53-BB79-950D853A1C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80CAC469-ADE8-49DF-9C28-AF10224B0F30}"/>
+  <xr:revisionPtr revIDLastSave="273" documentId="8_{CFF8497D-5AC5-4F53-BB79-950D853A1C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02CF813B-3E79-4F75-8CA3-3953FF9EBFF7}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3C2F71A7-BF18-485F-8BF5-EA2F93EB7B3B}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3C2F71A7-BF18-485F-8BF5-EA2F93EB7B3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
+    <sheet name="260427" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="44">
   <si>
     <t>Resultat efter finansiella poster:</t>
   </si>
@@ -151,6 +152,21 @@
   </si>
   <si>
     <t>När årsmötet har godkänt dispositionen så bokförs debet konto 2099 Åres resultat 434 975 kr, och kredit konto 2010 summa eget kapital.</t>
+  </si>
+  <si>
+    <t>Skillnad</t>
+  </si>
+  <si>
+    <t>kto 1300:</t>
+  </si>
+  <si>
+    <t>kto 1385:</t>
+  </si>
+  <si>
+    <t>Stiftelsevärdepapper:</t>
+  </si>
+  <si>
+    <t>"financial fixed assets, Securities":</t>
   </si>
 </sst>
 </file>
@@ -244,10 +260,6 @@
     </xf>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -259,12 +271,6 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -281,6 +287,14 @@
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -646,7 +660,7 @@
       <c r="D9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="16" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="10" t="s">
@@ -671,7 +685,7 @@
       <c r="D10" s="12">
         <v>-9507693</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="17">
         <v>881657</v>
       </c>
       <c r="F10" s="12">
@@ -692,7 +706,7 @@
       <c r="B11" s="11"/>
       <c r="C11" s="9"/>
       <c r="D11" s="12"/>
-      <c r="E11" s="19"/>
+      <c r="E11" s="17"/>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
       <c r="L11" s="2" t="s">
@@ -709,7 +723,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="12"/>
-      <c r="E12" s="19"/>
+      <c r="E12" s="17"/>
       <c r="F12" s="12">
         <f>1316633</f>
         <v>1316633</v>
@@ -726,7 +740,7 @@
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="20"/>
+      <c r="E13" s="18"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="L13" s="2"/>
@@ -735,7 +749,7 @@
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
-      <c r="E14" s="20"/>
+      <c r="E14" s="18"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="L14" s="3" t="s">
@@ -756,7 +770,7 @@
       <c r="D15" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="16" t="s">
         <v>8</v>
       </c>
       <c r="F15" s="10" t="s">
@@ -781,7 +795,7 @@
       <c r="D16" s="12">
         <v>-9507693</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="17">
         <f>-F18</f>
         <v>-434975.37</v>
       </c>
@@ -806,7 +820,7 @@
       <c r="B17" s="11"/>
       <c r="C17" s="9"/>
       <c r="D17" s="12"/>
-      <c r="E17" s="19"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
       <c r="L17" s="2" t="s">
@@ -822,7 +836,7 @@
         <v>11</v>
       </c>
       <c r="D18" s="12"/>
-      <c r="E18" s="19"/>
+      <c r="E18" s="17"/>
       <c r="F18" s="12">
         <f>M18</f>
         <v>434975.37</v>
@@ -849,7 +863,7 @@
     <row r="19" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
-      <c r="E19" s="20"/>
+      <c r="E19" s="18"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
     </row>
@@ -857,14 +871,14 @@
       <c r="B20" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="25"/>
-      <c r="D20" s="26" t="s">
+      <c r="C20" s="21"/>
+      <c r="D20" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="27" t="s">
+      <c r="E20" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="F20" s="26" t="s">
+      <c r="F20" s="22" t="s">
         <v>22</v>
       </c>
       <c r="G20" s="12"/>
@@ -876,7 +890,7 @@
       <c r="B21" s="8"/>
       <c r="C21" s="9"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="18"/>
+      <c r="E21" s="16"/>
       <c r="F21" s="13"/>
       <c r="G21" s="12"/>
       <c r="L21" s="2" t="s">
@@ -897,7 +911,7 @@
       <c r="D22" s="12">
         <v>-9507693</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="17">
         <v>0</v>
       </c>
       <c r="F22" s="12">
@@ -925,7 +939,7 @@
       <c r="D23" s="12">
         <v>0</v>
       </c>
-      <c r="E23" s="21">
+      <c r="E23" s="19">
         <f>-F18</f>
         <v>-434975.37</v>
       </c>
@@ -977,32 +991,32 @@
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B26" s="11"/>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D26" s="23"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
       <c r="G26" s="12"/>
       <c r="L26" s="2"/>
       <c r="M26" s="4"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B27" s="11"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
       <c r="G27" s="12"/>
       <c r="L27" s="2"/>
       <c r="M27" s="4"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B28" s="11"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
       <c r="G28" s="12"/>
       <c r="L28" s="2"/>
       <c r="M28" s="4"/>
@@ -1013,7 +1027,7 @@
         <v>14</v>
       </c>
       <c r="D29" s="12"/>
-      <c r="E29" s="21"/>
+      <c r="E29" s="19"/>
       <c r="F29" s="12">
         <f>-113186</f>
         <v>-113186</v>
@@ -1028,7 +1042,7 @@
       <c r="B30" s="11"/>
       <c r="C30" s="9"/>
       <c r="D30" s="12"/>
-      <c r="E30" s="21"/>
+      <c r="E30" s="19"/>
       <c r="F30" s="12"/>
       <c r="G30" s="12"/>
       <c r="L30" s="2"/>
@@ -1050,11 +1064,8 @@
       <c r="L31" s="2"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B32" s="16"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="16"/>
+      <c r="C32" s="2"/>
+      <c r="E32" s="2"/>
     </row>
     <row r="33" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" s="11"/>
@@ -1111,7 +1122,7 @@
       <c r="C39" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D39" s="28" t="s">
+      <c r="D39" s="24" t="s">
         <v>26</v>
       </c>
       <c r="E39" s="11"/>
@@ -1176,6 +1187,771 @@
       <c r="D45" s="11"/>
       <c r="E45" s="11"/>
       <c r="F45" s="11"/>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <mergeCells count="1">
+    <mergeCell ref="C26:F27"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42EA386F-145E-494F-8F9B-8833E25F5D8C}">
+  <dimension ref="B3:N59"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="42.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="43.42578125" customWidth="1"/>
+    <col min="10" max="10" width="24.5703125" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="M3" s="1"/>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="L4" s="2"/>
+      <c r="M4" s="1"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="L5" s="2"/>
+      <c r="M5" s="1">
+        <v>1316632</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="L6" s="2"/>
+      <c r="M6" s="1">
+        <v>881657</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="L7" s="2"/>
+      <c r="M7" s="1">
+        <f>M5-M6</f>
+        <v>434975</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="E8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="1"/>
+    </row>
+    <row r="9" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="M9" s="1">
+        <v>1300704</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B10" s="11"/>
+      <c r="C10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="E10" s="17">
+        <v>881657</v>
+      </c>
+      <c r="F10" s="12">
+        <f>D10+E10</f>
+        <v>-8626036</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="M10" s="1">
+        <v>-881657</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B11" s="11"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="L11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M11" s="1">
+        <f>M9+M10</f>
+        <v>419047</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B12" s="11"/>
+      <c r="C12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="12"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="12">
+        <f>1316633</f>
+        <v>1316633</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L12" s="2"/>
+      <c r="M12" s="1"/>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C13" s="2"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="4"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C14" s="2"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="L14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="M14" s="4">
+        <v>35303.4</v>
+      </c>
+      <c r="N14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" s="12"/>
+      <c r="L15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M15" s="4">
+        <v>578936.24</v>
+      </c>
+      <c r="N15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B16" s="11"/>
+      <c r="C16" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="E16" s="17">
+        <f>-F18</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="F16" s="12">
+        <f>D16+E16</f>
+        <v>-9942668.3699999992</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M16" s="4">
+        <v>-195193</v>
+      </c>
+      <c r="N16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B17" s="11"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="L17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M17" s="4">
+        <v>15928.73</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B18" s="11"/>
+      <c r="C18" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="12"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="12">
+        <f>M18</f>
+        <v>434975.37</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" t="s">
+        <v>30</v>
+      </c>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="M18" s="7">
+        <f>SUM(M14:M17)</f>
+        <v>434975.37</v>
+      </c>
+      <c r="N18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C19" s="2"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="21"/>
+      <c r="D20" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="12"/>
+      <c r="H20" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B21" s="8"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="12"/>
+      <c r="L21" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="M21" s="4">
+        <v>881657</v>
+      </c>
+      <c r="N21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B22" s="11"/>
+      <c r="C22" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="E22" s="17">
+        <v>0</v>
+      </c>
+      <c r="F22" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="M22" s="4">
+        <f>SUM(M18:M21)</f>
+        <v>1316632.3700000001</v>
+      </c>
+      <c r="N22" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B23" s="11"/>
+      <c r="C23" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="12">
+        <v>0</v>
+      </c>
+      <c r="E23" s="19">
+        <f>-F18</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="F23" s="12">
+        <f>D23+E23</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H23" t="s">
+        <v>33</v>
+      </c>
+      <c r="L23" s="2"/>
+      <c r="M23" s="4"/>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B24" s="11"/>
+      <c r="C24" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="14">
+        <f>SUM(D22:D23)</f>
+        <v>-9507693</v>
+      </c>
+      <c r="E24" s="14">
+        <f>SUM(E22:E23)</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="F24" s="14">
+        <f>SUM(F22:F23)</f>
+        <v>-9942668.3699999992</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L24" s="2"/>
+      <c r="M24" s="4"/>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B25" s="11"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="12"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="4"/>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B26" s="11"/>
+      <c r="C26" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="12"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="4"/>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B27" s="11"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="12"/>
+      <c r="L27" s="2"/>
+      <c r="M27" s="4"/>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B28" s="11"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="12"/>
+      <c r="L28" s="2"/>
+      <c r="M28" s="4"/>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B29" s="11"/>
+      <c r="C29" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="12"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="12">
+        <f>-113186</f>
+        <v>-113186</v>
+      </c>
+      <c r="G29" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L29" s="2"/>
+      <c r="M29" s="4"/>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B30" s="11"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="L30" s="2"/>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B31" s="11"/>
+      <c r="C31" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="14">
+        <f>SUM(F24:F30)</f>
+        <v>-10055854.369999999</v>
+      </c>
+      <c r="G31" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L31" s="2"/>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C32" s="2"/>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="11"/>
+      <c r="C33" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="12">
+        <f>10055854+F31</f>
+        <v>-0.36999999918043613</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H33" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B35" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
+    </row>
+    <row r="36" spans="2:8" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="15"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+    </row>
+    <row r="37" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B37" s="11"/>
+      <c r="C37" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+    </row>
+    <row r="38" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="11"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="11"/>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B39" s="11"/>
+      <c r="C39" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D39" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="E39" s="11"/>
+      <c r="F39" s="11"/>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B40" s="11"/>
+      <c r="C40" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40" s="12">
+        <v>9507693</v>
+      </c>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B41" s="11"/>
+      <c r="C41" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" s="12">
+        <f>F18</f>
+        <v>434975.37</v>
+      </c>
+      <c r="E41" s="11"/>
+      <c r="F41" s="11"/>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B42" s="11"/>
+      <c r="C42" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D42" s="14">
+        <f>SUM(D40:D41)</f>
+        <v>9942668.3699999992</v>
+      </c>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B43" s="11"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="11"/>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B44" s="11"/>
+      <c r="C44" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="11"/>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B45" s="11"/>
+      <c r="C45" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="11"/>
+    </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B49" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" s="11"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="11"/>
+    </row>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B50" s="15"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="11"/>
+      <c r="J50" s="2"/>
+      <c r="L50" s="28">
+        <v>46138</v>
+      </c>
+      <c r="M50" s="28">
+        <v>46139</v>
+      </c>
+    </row>
+    <row r="51" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B51" s="11"/>
+      <c r="C51" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D51" s="11"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="11"/>
+      <c r="J51" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L51" s="4">
+        <v>444505</v>
+      </c>
+      <c r="M51" s="4">
+        <v>451336.33</v>
+      </c>
+      <c r="N51" s="4">
+        <f>M51-L51</f>
+        <v>6831.3300000000163</v>
+      </c>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B52" s="11"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="27">
+        <v>46138</v>
+      </c>
+      <c r="E52" s="11"/>
+      <c r="F52" s="27">
+        <v>46139</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L52" s="4">
+        <v>8632426.8900000006</v>
+      </c>
+      <c r="M52" s="4">
+        <v>8845883.5199999996</v>
+      </c>
+      <c r="N52" s="4">
+        <f>M52-L52</f>
+        <v>213456.62999999896</v>
+      </c>
+    </row>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B53" s="11"/>
+      <c r="C53" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D53" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="E53" s="11"/>
+      <c r="F53" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="7">
+        <f>SUM(N51:N52)</f>
+        <v>220287.95999999897</v>
+      </c>
+    </row>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B54" s="11"/>
+      <c r="C54" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D54" s="12">
+        <v>9507693</v>
+      </c>
+      <c r="E54" s="11"/>
+      <c r="F54" s="12">
+        <v>9507693</v>
+      </c>
+      <c r="J54" s="2"/>
+    </row>
+    <row r="55" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B55" s="11"/>
+      <c r="C55" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D55" s="12">
+        <f>424975.37</f>
+        <v>424975.37</v>
+      </c>
+      <c r="E55" s="11"/>
+      <c r="F55" s="12">
+        <f>645262.92</f>
+        <v>645262.92000000004</v>
+      </c>
+      <c r="H55" s="1">
+        <f>F55-D55</f>
+        <v>220287.55000000005</v>
+      </c>
+      <c r="J55" s="2"/>
+    </row>
+    <row r="56" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B56" s="11"/>
+      <c r="C56" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D56" s="14">
+        <f>SUM(D54:D55)</f>
+        <v>9932668.3699999992</v>
+      </c>
+      <c r="E56" s="11"/>
+      <c r="F56" s="14">
+        <f>SUM(F54:F55)</f>
+        <v>10152955.92</v>
+      </c>
+    </row>
+    <row r="57" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B57" s="11"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+    </row>
+    <row r="58" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B58" s="11"/>
+      <c r="C58" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+    </row>
+    <row r="59" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B59" s="11"/>
+      <c r="C59" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Update CLAUDE.md to version 4.6, reflecting the latest revisions for audit instructions, including new guidelines on reporting changes in equity and ensuring correct titling of financial statements. Added a new PDF document for the 2025 financial statements, ensuring compliance with reporting standards. Updated version indicators to reflect the latest changes as of 2026-04-29.
</commit_message>
<xml_diff>
--- a/KalmarNation/revision/_egen_analys/Egen_analys.xlsx
+++ b/KalmarNation/revision/_egen_analys/Egen_analys.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/ClaudeCowork/KalmarNation/revision/_egen_analys/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="273" documentId="8_{CFF8497D-5AC5-4F53-BB79-950D853A1C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02CF813B-3E79-4F75-8CA3-3953FF9EBFF7}"/>
+  <xr:revisionPtr revIDLastSave="284" documentId="8_{CFF8497D-5AC5-4F53-BB79-950D853A1C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D6E1244-F47E-45F2-9BDE-4C0627CC9E0D}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3C2F71A7-BF18-485F-8BF5-EA2F93EB7B3B}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3C2F71A7-BF18-485F-8BF5-EA2F93EB7B3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
     <sheet name="260427" sheetId="2" r:id="rId2"/>
+    <sheet name="260429" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="45">
   <si>
     <t>Resultat efter finansiella poster:</t>
   </si>
@@ -167,6 +168,9 @@
   </si>
   <si>
     <t>"financial fixed assets, Securities":</t>
+  </si>
+  <si>
+    <t>Resultat</t>
   </si>
 </sst>
 </file>
@@ -205,7 +209,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -215,6 +219,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -231,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -295,6 +305,8 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -310,6 +322,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>303969</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>171221</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Bildobjekt 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E1337E4-0796-CDB0-4775-2EE3D99B43F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7381875" y="6210300"/>
+          <a:ext cx="6647619" cy="1828571"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1959,4 +2020,785 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C30379D-5427-4A85-83BA-D338278EB380}">
+  <dimension ref="B3:N59"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="42.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="43.42578125" customWidth="1"/>
+    <col min="10" max="10" width="24.5703125" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="M3" s="1"/>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="L4" s="2"/>
+      <c r="M4" s="1"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="L5" s="2"/>
+      <c r="M5" s="1">
+        <v>1316632</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="L6" s="2"/>
+      <c r="M6" s="1">
+        <v>881657</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="L7" s="2"/>
+      <c r="M7" s="1">
+        <f>M5-M6</f>
+        <v>434975</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="E8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="1"/>
+    </row>
+    <row r="9" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="M9" s="1">
+        <v>1300704</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B10" s="11"/>
+      <c r="C10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="E10" s="17">
+        <v>881657</v>
+      </c>
+      <c r="F10" s="12">
+        <f>D10+E10</f>
+        <v>-8626036</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="M10" s="1">
+        <v>-881657</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B11" s="11"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="L11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M11" s="1">
+        <f>M9+M10</f>
+        <v>419047</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B12" s="11"/>
+      <c r="C12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="12"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="12">
+        <f>1316633</f>
+        <v>1316633</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L12" s="2"/>
+      <c r="M12" s="1"/>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C13" s="2"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="4"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C14" s="2"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="L14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="M14" s="4">
+        <v>35303.4</v>
+      </c>
+      <c r="N14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" s="12"/>
+      <c r="L15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M15" s="4">
+        <v>578936.24</v>
+      </c>
+      <c r="N15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B16" s="11"/>
+      <c r="C16" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="E16" s="17">
+        <f>-F18</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="F16" s="12">
+        <f>D16+E16</f>
+        <v>-9942668.3699999992</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M16" s="4">
+        <v>-195193</v>
+      </c>
+      <c r="N16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B17" s="11"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="L17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M17" s="4">
+        <v>15928.73</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B18" s="11"/>
+      <c r="C18" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="12"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="12">
+        <f>M18</f>
+        <v>434975.37</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" t="s">
+        <v>30</v>
+      </c>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="M18" s="7">
+        <f>SUM(M14:M17)</f>
+        <v>434975.37</v>
+      </c>
+      <c r="N18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C19" s="2"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="21"/>
+      <c r="D20" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="12"/>
+      <c r="H20" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B21" s="8"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="12"/>
+      <c r="L21" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="M21" s="4">
+        <v>881657</v>
+      </c>
+      <c r="N21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B22" s="11"/>
+      <c r="C22" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="E22" s="17">
+        <v>0</v>
+      </c>
+      <c r="F22" s="12">
+        <v>-9507693</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="M22" s="4">
+        <f>SUM(M18:M21)</f>
+        <v>1316632.3700000001</v>
+      </c>
+      <c r="N22" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B23" s="11"/>
+      <c r="C23" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="12">
+        <v>0</v>
+      </c>
+      <c r="E23" s="19">
+        <f>-F18</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="F23" s="12">
+        <f>D23+E23</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H23" t="s">
+        <v>33</v>
+      </c>
+      <c r="L23" s="2"/>
+      <c r="M23" s="4"/>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B24" s="11"/>
+      <c r="C24" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="14">
+        <f>SUM(D22:D23)</f>
+        <v>-9507693</v>
+      </c>
+      <c r="E24" s="14">
+        <f>SUM(E22:E23)</f>
+        <v>-434975.37</v>
+      </c>
+      <c r="F24" s="14">
+        <f>SUM(F22:F23)</f>
+        <v>-9942668.3699999992</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L24" s="2"/>
+      <c r="M24" s="4"/>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B25" s="11"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="12"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="4"/>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B26" s="11"/>
+      <c r="C26" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="12"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="4"/>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B27" s="11"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="12"/>
+      <c r="L27" s="2"/>
+      <c r="M27" s="4"/>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B28" s="11"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="12"/>
+      <c r="L28" s="2"/>
+      <c r="M28" s="4"/>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B29" s="11"/>
+      <c r="C29" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="12"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="12">
+        <f>-113186</f>
+        <v>-113186</v>
+      </c>
+      <c r="G29" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L29" s="2"/>
+      <c r="M29" s="4"/>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B30" s="11"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="L30" s="2"/>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B31" s="11"/>
+      <c r="C31" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="14">
+        <f>SUM(F24:F30)</f>
+        <v>-10055854.369999999</v>
+      </c>
+      <c r="G31" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L31" s="2"/>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C32" s="2"/>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="11"/>
+      <c r="C33" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="12">
+        <f>10055854+F31</f>
+        <v>-0.36999999918043613</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H33" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B35" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
+    </row>
+    <row r="36" spans="2:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="15"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+    </row>
+    <row r="37" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B37" s="11"/>
+      <c r="C37" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+    </row>
+    <row r="38" spans="2:12" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="11"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="11"/>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B39" s="11"/>
+      <c r="C39" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D39" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="E39" s="11"/>
+      <c r="F39" s="11"/>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B40" s="11"/>
+      <c r="C40" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40" s="12">
+        <v>9507693</v>
+      </c>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B41" s="11"/>
+      <c r="C41" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" s="12">
+        <f>F18</f>
+        <v>434975.37</v>
+      </c>
+      <c r="E41" s="11"/>
+      <c r="F41" s="11"/>
+    </row>
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B42" s="11"/>
+      <c r="C42" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D42" s="14">
+        <f>SUM(D40:D41)</f>
+        <v>9942668.3699999992</v>
+      </c>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+    </row>
+    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B43" s="11"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="11"/>
+    </row>
+    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B44" s="11"/>
+      <c r="C44" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="11"/>
+    </row>
+    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B45" s="11"/>
+      <c r="C45" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="11"/>
+      <c r="L45" s="29" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J46" s="1">
+        <v>10152956.050000001</v>
+      </c>
+      <c r="K46" s="1">
+        <v>9507693.0999999996</v>
+      </c>
+      <c r="L46" s="30">
+        <f>J46-K46</f>
+        <v>645262.95000000112</v>
+      </c>
+    </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B49" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" s="11"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="11"/>
+    </row>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B50" s="15"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="11"/>
+      <c r="J50" s="2"/>
+      <c r="L50" s="28">
+        <v>46138</v>
+      </c>
+      <c r="M50" s="28">
+        <v>46139</v>
+      </c>
+    </row>
+    <row r="51" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B51" s="11"/>
+      <c r="C51" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D51" s="11"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="11"/>
+      <c r="J51" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L51" s="4">
+        <v>444505</v>
+      </c>
+      <c r="M51" s="4">
+        <v>451336.33</v>
+      </c>
+      <c r="N51" s="4">
+        <f>M51-L51</f>
+        <v>6831.3300000000163</v>
+      </c>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B52" s="11"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="27">
+        <v>46138</v>
+      </c>
+      <c r="E52" s="11"/>
+      <c r="F52" s="27">
+        <v>46139</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L52" s="4">
+        <v>8632426.8900000006</v>
+      </c>
+      <c r="M52" s="4">
+        <v>8845883.5199999996</v>
+      </c>
+      <c r="N52" s="4">
+        <f>M52-L52</f>
+        <v>213456.62999999896</v>
+      </c>
+    </row>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B53" s="11"/>
+      <c r="C53" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D53" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="E53" s="11"/>
+      <c r="F53" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="7">
+        <f>SUM(N51:N52)</f>
+        <v>220287.95999999897</v>
+      </c>
+    </row>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B54" s="11"/>
+      <c r="C54" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D54" s="12">
+        <v>9507693</v>
+      </c>
+      <c r="E54" s="11"/>
+      <c r="F54" s="12">
+        <v>9507693</v>
+      </c>
+      <c r="J54" s="2"/>
+    </row>
+    <row r="55" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B55" s="11"/>
+      <c r="C55" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D55" s="12">
+        <f>424975.37</f>
+        <v>424975.37</v>
+      </c>
+      <c r="E55" s="11"/>
+      <c r="F55" s="12">
+        <f>645262.92</f>
+        <v>645262.92000000004</v>
+      </c>
+      <c r="H55" s="1">
+        <f>F55-D55</f>
+        <v>220287.55000000005</v>
+      </c>
+      <c r="J55" s="2"/>
+    </row>
+    <row r="56" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B56" s="11"/>
+      <c r="C56" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D56" s="14">
+        <f>SUM(D54:D55)</f>
+        <v>9932668.3699999992</v>
+      </c>
+      <c r="E56" s="11"/>
+      <c r="F56" s="14">
+        <f>SUM(F54:F55)</f>
+        <v>10152955.92</v>
+      </c>
+    </row>
+    <row r="57" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B57" s="11"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+    </row>
+    <row r="58" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B58" s="11"/>
+      <c r="C58" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+    </row>
+    <row r="59" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B59" s="11"/>
+      <c r="C59" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C26:F27"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>